<commit_message>
Fix CV export template picture replacement
</commit_message>
<xml_diff>
--- a/public/templates/cv-form-new-ver.xlsx
+++ b/public/templates/cv-form-new-ver.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\KMT\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A489B5DB-5015-4AAD-B9EC-F69AD391E30E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9F5BC75-BD5C-4BD1-84FB-80158F9AB30C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="68">
   <si>
     <t>PERSON'S DETAILS :</t>
   </si>
@@ -240,6 +240,12 @@
   </si>
   <si>
     <t>Picture</t>
+  </si>
+  <si>
+    <t>CERTIFICATE OF COMPETENCY:</t>
+  </si>
+  <si>
+    <t>CERTIFICATE OF COMPETENCY</t>
   </si>
 </sst>
 </file>
@@ -553,18 +559,18 @@
     <xf numFmtId="15" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -574,20 +580,20 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -607,24 +613,24 @@
     <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="15" fontId="5" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -637,6 +643,24 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -657,24 +681,6 @@
     </xf>
     <xf numFmtId="15" fontId="5" fillId="0" borderId="15" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -691,6 +697,62 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>45522</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>32657</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>891393</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>304800</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B7AFCB3E-870E-263A-D43C-AC6B96BE4B02}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="26806" r="27917" b="66333"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8394865" y="576943"/>
+          <a:ext cx="1814699" cy="2362200"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -979,118 +1041,118 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
     </row>
     <row r="3" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="41" t="s">
+      <c r="A3" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="42"/>
-      <c r="C3" s="43"/>
-      <c r="D3" s="44"/>
-      <c r="E3" s="44"/>
-      <c r="F3" s="41" t="s">
+      <c r="B3" s="40"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="42"/>
+      <c r="E3" s="42"/>
+      <c r="F3" s="39" t="s">
         <v>32</v>
       </c>
-      <c r="G3" s="42"/>
-      <c r="H3" s="43"/>
-      <c r="I3" s="44"/>
-      <c r="J3" s="44"/>
-      <c r="K3" s="44"/>
-      <c r="L3" s="56" t="s">
+      <c r="G3" s="40"/>
+      <c r="H3" s="41"/>
+      <c r="I3" s="42"/>
+      <c r="J3" s="42"/>
+      <c r="K3" s="42"/>
+      <c r="L3" s="49" t="s">
         <v>65</v>
       </c>
-      <c r="M3" s="57"/>
+      <c r="M3" s="50"/>
     </row>
     <row r="4" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="41" t="s">
+      <c r="A4" s="39" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="42"/>
-      <c r="C4" s="43"/>
-      <c r="D4" s="44"/>
-      <c r="E4" s="44"/>
-      <c r="F4" s="41" t="s">
+      <c r="B4" s="40"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="42"/>
+      <c r="E4" s="42"/>
+      <c r="F4" s="39" t="s">
         <v>27</v>
       </c>
-      <c r="G4" s="42"/>
-      <c r="H4" s="43"/>
-      <c r="I4" s="44"/>
-      <c r="J4" s="44"/>
-      <c r="K4" s="44"/>
-      <c r="L4" s="58"/>
-      <c r="M4" s="59"/>
+      <c r="G4" s="40"/>
+      <c r="H4" s="41"/>
+      <c r="I4" s="42"/>
+      <c r="J4" s="42"/>
+      <c r="K4" s="42"/>
+      <c r="L4" s="51"/>
+      <c r="M4" s="52"/>
     </row>
     <row r="5" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="41" t="s">
+      <c r="A5" s="39" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="42"/>
-      <c r="C5" s="52"/>
-      <c r="D5" s="53"/>
-      <c r="E5" s="54"/>
-      <c r="F5" s="41" t="s">
+      <c r="B5" s="40"/>
+      <c r="C5" s="58"/>
+      <c r="D5" s="59"/>
+      <c r="E5" s="60"/>
+      <c r="F5" s="39" t="s">
         <v>33</v>
       </c>
-      <c r="G5" s="42"/>
-      <c r="H5" s="43"/>
-      <c r="I5" s="44"/>
-      <c r="J5" s="44"/>
-      <c r="K5" s="44"/>
-      <c r="L5" s="58"/>
-      <c r="M5" s="59"/>
+      <c r="G5" s="40"/>
+      <c r="H5" s="41"/>
+      <c r="I5" s="42"/>
+      <c r="J5" s="42"/>
+      <c r="K5" s="42"/>
+      <c r="L5" s="51"/>
+      <c r="M5" s="52"/>
     </row>
     <row r="6" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="41" t="s">
+      <c r="A6" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="42"/>
+      <c r="B6" s="40"/>
       <c r="C6" s="45"/>
-      <c r="D6" s="55"/>
+      <c r="D6" s="61"/>
       <c r="E6" s="46"/>
-      <c r="F6" s="41" t="s">
+      <c r="F6" s="39" t="s">
         <v>34</v>
       </c>
-      <c r="G6" s="42"/>
-      <c r="H6" s="43"/>
-      <c r="I6" s="44"/>
-      <c r="J6" s="44"/>
-      <c r="K6" s="44"/>
-      <c r="L6" s="58"/>
-      <c r="M6" s="59"/>
+      <c r="G6" s="40"/>
+      <c r="H6" s="41"/>
+      <c r="I6" s="42"/>
+      <c r="J6" s="42"/>
+      <c r="K6" s="42"/>
+      <c r="L6" s="51"/>
+      <c r="M6" s="52"/>
     </row>
     <row r="7" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="41" t="s">
+      <c r="A7" s="39" t="s">
         <v>39</v>
       </c>
-      <c r="B7" s="42"/>
-      <c r="C7" s="43"/>
-      <c r="D7" s="44"/>
-      <c r="E7" s="44"/>
-      <c r="F7" s="49" t="s">
+      <c r="B7" s="40"/>
+      <c r="C7" s="41"/>
+      <c r="D7" s="42"/>
+      <c r="E7" s="42"/>
+      <c r="F7" s="55" t="s">
         <v>40</v>
       </c>
-      <c r="G7" s="50"/>
-      <c r="H7" s="51"/>
-      <c r="I7" s="44"/>
-      <c r="J7" s="44"/>
-      <c r="K7" s="44"/>
-      <c r="L7" s="58"/>
-      <c r="M7" s="59"/>
+      <c r="G7" s="56"/>
+      <c r="H7" s="57"/>
+      <c r="I7" s="42"/>
+      <c r="J7" s="42"/>
+      <c r="K7" s="42"/>
+      <c r="L7" s="51"/>
+      <c r="M7" s="52"/>
     </row>
     <row r="8" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="41" t="s">
+      <c r="A8" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="42"/>
-      <c r="C8" s="43"/>
-      <c r="D8" s="44"/>
-      <c r="E8" s="44"/>
+      <c r="B8" s="40"/>
+      <c r="C8" s="41"/>
+      <c r="D8" s="42"/>
+      <c r="E8" s="42"/>
       <c r="F8" s="9" t="s">
         <v>35</v>
       </c>
@@ -1101,17 +1163,17 @@
       </c>
       <c r="J8" s="45"/>
       <c r="K8" s="46"/>
-      <c r="L8" s="58"/>
-      <c r="M8" s="59"/>
+      <c r="L8" s="51"/>
+      <c r="M8" s="52"/>
     </row>
     <row r="9" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="41" t="s">
+      <c r="A9" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="42"/>
-      <c r="C9" s="43"/>
-      <c r="D9" s="44"/>
-      <c r="E9" s="44"/>
+      <c r="B9" s="40"/>
+      <c r="C9" s="41"/>
+      <c r="D9" s="42"/>
+      <c r="E9" s="42"/>
       <c r="F9" s="9" t="s">
         <v>35</v>
       </c>
@@ -1122,38 +1184,38 @@
       </c>
       <c r="J9" s="45"/>
       <c r="K9" s="46"/>
-      <c r="L9" s="60"/>
-      <c r="M9" s="61"/>
+      <c r="L9" s="53"/>
+      <c r="M9" s="54"/>
     </row>
     <row r="10" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="41" t="s">
+      <c r="A10" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="B10" s="42"/>
+      <c r="B10" s="40"/>
       <c r="C10" s="47"/>
-      <c r="D10" s="44"/>
-      <c r="E10" s="44"/>
+      <c r="D10" s="42"/>
+      <c r="E10" s="42"/>
       <c r="F10" s="9" t="s">
         <v>35</v>
       </c>
       <c r="G10" s="48"/>
-      <c r="H10" s="43"/>
+      <c r="H10" s="41"/>
       <c r="I10" s="5"/>
       <c r="J10" s="5"/>
       <c r="K10" s="5"/>
     </row>
     <row r="12" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="28" t="s">
-        <v>28</v>
-      </c>
-      <c r="B12" s="28"/>
-      <c r="C12" s="28"/>
-      <c r="D12" s="28"/>
-      <c r="E12" s="28"/>
+      <c r="A12" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="B12" s="31"/>
+      <c r="C12" s="31"/>
+      <c r="D12" s="31"/>
+      <c r="E12" s="31"/>
     </row>
     <row r="14" spans="1:13" s="7" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="36" t="s">
-        <v>29</v>
+        <v>67</v>
       </c>
       <c r="B14" s="36"/>
       <c r="C14" s="36"/>
@@ -1162,10 +1224,10 @@
         <v>30</v>
       </c>
       <c r="F14" s="26"/>
-      <c r="G14" s="39" t="s">
+      <c r="G14" s="43" t="s">
         <v>31</v>
       </c>
-      <c r="H14" s="40"/>
+      <c r="H14" s="44"/>
       <c r="I14" s="26" t="s">
         <v>11</v>
       </c>
@@ -1209,12 +1271,12 @@
       <c r="M16" s="18"/>
     </row>
     <row r="18" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="28" t="s">
+      <c r="A18" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="B18" s="28"/>
-      <c r="C18" s="28"/>
-      <c r="D18" s="28"/>
+      <c r="B18" s="31"/>
+      <c r="C18" s="31"/>
+      <c r="D18" s="31"/>
     </row>
     <row r="20" spans="1:13" s="3" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="26" t="s">
@@ -1222,20 +1284,20 @@
       </c>
       <c r="B20" s="26"/>
       <c r="C20" s="26"/>
-      <c r="D20" s="24" t="s">
+      <c r="D20" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="E20" s="24"/>
-      <c r="F20" s="24"/>
-      <c r="G20" s="24"/>
-      <c r="H20" s="24"/>
-      <c r="I20" s="24" t="s">
+      <c r="E20" s="22"/>
+      <c r="F20" s="22"/>
+      <c r="G20" s="22"/>
+      <c r="H20" s="22"/>
+      <c r="I20" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="J20" s="24"/>
-      <c r="K20" s="24"/>
-      <c r="L20" s="24"/>
-      <c r="M20" s="24"/>
+      <c r="J20" s="22"/>
+      <c r="K20" s="22"/>
+      <c r="L20" s="22"/>
+      <c r="M20" s="22"/>
     </row>
     <row r="21" spans="1:13" s="3" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="26"/>
@@ -1509,149 +1571,137 @@
       <c r="M37" s="8"/>
     </row>
     <row r="38" spans="1:13" ht="26.4" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="28" t="s">
+      <c r="A38" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="B38" s="28"/>
-      <c r="C38" s="28"/>
-      <c r="D38" s="28"/>
-      <c r="E38" s="28"/>
+      <c r="B38" s="31"/>
+      <c r="C38" s="31"/>
+      <c r="D38" s="31"/>
+      <c r="E38" s="31"/>
     </row>
     <row r="40" spans="1:13" s="3" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="24" t="s">
+      <c r="A40" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="B40" s="24"/>
-      <c r="C40" s="24"/>
-      <c r="D40" s="24"/>
-      <c r="E40" s="24" t="s">
+      <c r="B40" s="22"/>
+      <c r="C40" s="22"/>
+      <c r="D40" s="22"/>
+      <c r="E40" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="F40" s="24"/>
-      <c r="G40" s="24" t="s">
+      <c r="F40" s="22"/>
+      <c r="G40" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="H40" s="24"/>
-      <c r="I40" s="24"/>
-      <c r="J40" s="24" t="s">
+      <c r="H40" s="22"/>
+      <c r="I40" s="22"/>
+      <c r="J40" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="K40" s="24"/>
-      <c r="L40" s="24" t="s">
+      <c r="K40" s="22"/>
+      <c r="L40" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="M40" s="24"/>
+      <c r="M40" s="22"/>
     </row>
     <row r="41" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="29" t="s">
+      <c r="A41" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="B41" s="29"/>
-      <c r="C41" s="29"/>
-      <c r="D41" s="29"/>
-      <c r="E41" s="30"/>
-      <c r="F41" s="30"/>
-      <c r="G41" s="31"/>
-      <c r="H41" s="31"/>
-      <c r="I41" s="31"/>
-      <c r="J41" s="32"/>
-      <c r="K41" s="32"/>
-      <c r="L41" s="32"/>
-      <c r="M41" s="32"/>
+      <c r="B41" s="28"/>
+      <c r="C41" s="28"/>
+      <c r="D41" s="28"/>
+      <c r="E41" s="32"/>
+      <c r="F41" s="32"/>
+      <c r="G41" s="29"/>
+      <c r="H41" s="29"/>
+      <c r="I41" s="29"/>
+      <c r="J41" s="30"/>
+      <c r="K41" s="30"/>
+      <c r="L41" s="30"/>
+      <c r="M41" s="30"/>
     </row>
     <row r="42" spans="1:13" ht="40.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="29" t="s">
+      <c r="A42" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="B42" s="29"/>
-      <c r="C42" s="29"/>
-      <c r="D42" s="29"/>
-      <c r="E42" s="31"/>
-      <c r="F42" s="31"/>
-      <c r="G42" s="31"/>
-      <c r="H42" s="31"/>
-      <c r="I42" s="31"/>
-      <c r="J42" s="32"/>
-      <c r="K42" s="32"/>
-      <c r="L42" s="32"/>
-      <c r="M42" s="32"/>
+      <c r="B42" s="28"/>
+      <c r="C42" s="28"/>
+      <c r="D42" s="28"/>
+      <c r="E42" s="29"/>
+      <c r="F42" s="29"/>
+      <c r="G42" s="29"/>
+      <c r="H42" s="29"/>
+      <c r="I42" s="29"/>
+      <c r="J42" s="30"/>
+      <c r="K42" s="30"/>
+      <c r="L42" s="30"/>
+      <c r="M42" s="30"/>
     </row>
     <row r="43" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="28" t="s">
+      <c r="A43" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="B43" s="28"/>
-      <c r="C43" s="28"/>
-      <c r="D43" s="28"/>
+      <c r="B43" s="31"/>
+      <c r="C43" s="31"/>
+      <c r="D43" s="31"/>
     </row>
     <row r="45" spans="1:13" s="3" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="24" t="s">
+      <c r="A45" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="B45" s="24"/>
-      <c r="C45" s="24"/>
-      <c r="D45" s="24"/>
-      <c r="E45" s="24" t="s">
+      <c r="B45" s="22"/>
+      <c r="C45" s="22"/>
+      <c r="D45" s="22"/>
+      <c r="E45" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="F45" s="24"/>
-      <c r="G45" s="24"/>
-      <c r="H45" s="24" t="s">
+      <c r="F45" s="22"/>
+      <c r="G45" s="22"/>
+      <c r="H45" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="I45" s="24"/>
-      <c r="J45" s="24"/>
-      <c r="K45" s="24" t="s">
+      <c r="I45" s="22"/>
+      <c r="J45" s="22"/>
+      <c r="K45" s="22" t="s">
         <v>37</v>
       </c>
-      <c r="L45" s="24"/>
-      <c r="M45" s="24"/>
+      <c r="L45" s="22"/>
+      <c r="M45" s="22"/>
     </row>
     <row r="46" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="23" t="s">
+      <c r="A46" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="B46" s="23"/>
-      <c r="C46" s="23"/>
-      <c r="D46" s="23"/>
-      <c r="E46" s="24" t="s">
-        <v>42</v>
-      </c>
-      <c r="F46" s="24"/>
-      <c r="G46" s="24"/>
-      <c r="H46" s="24" t="s">
-        <v>42</v>
-      </c>
-      <c r="I46" s="24"/>
-      <c r="J46" s="24"/>
-      <c r="K46" s="24" t="s">
-        <v>42</v>
-      </c>
-      <c r="L46" s="24"/>
-      <c r="M46" s="24"/>
+      <c r="B46" s="21"/>
+      <c r="C46" s="21"/>
+      <c r="D46" s="21"/>
+      <c r="E46" s="22"/>
+      <c r="F46" s="22"/>
+      <c r="G46" s="22"/>
+      <c r="H46" s="22"/>
+      <c r="I46" s="22"/>
+      <c r="J46" s="22"/>
+      <c r="K46" s="22"/>
+      <c r="L46" s="22"/>
+      <c r="M46" s="22"/>
     </row>
     <row r="47" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="23" t="s">
+      <c r="A47" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="B47" s="23"/>
-      <c r="C47" s="23"/>
-      <c r="D47" s="23"/>
-      <c r="E47" s="24" t="s">
-        <v>42</v>
-      </c>
-      <c r="F47" s="24"/>
-      <c r="G47" s="24"/>
-      <c r="H47" s="24" t="s">
-        <v>42</v>
-      </c>
-      <c r="I47" s="24"/>
-      <c r="J47" s="24"/>
-      <c r="K47" s="24" t="s">
-        <v>42</v>
-      </c>
-      <c r="L47" s="24"/>
-      <c r="M47" s="24"/>
+      <c r="B47" s="21"/>
+      <c r="C47" s="21"/>
+      <c r="D47" s="21"/>
+      <c r="E47" s="22"/>
+      <c r="F47" s="22"/>
+      <c r="G47" s="22"/>
+      <c r="H47" s="22"/>
+      <c r="I47" s="22"/>
+      <c r="J47" s="22"/>
+      <c r="K47" s="22"/>
+      <c r="L47" s="22"/>
+      <c r="M47" s="22"/>
     </row>
     <row r="49" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="25" t="s">
@@ -1714,8 +1764,8 @@
       <c r="G52" s="15"/>
       <c r="H52" s="19"/>
       <c r="I52" s="20"/>
-      <c r="J52" s="21"/>
-      <c r="K52" s="22"/>
+      <c r="J52" s="23"/>
+      <c r="K52" s="24"/>
       <c r="L52" s="15"/>
       <c r="M52" s="15"/>
     </row>
@@ -2230,7 +2280,8 @@
   <headerFooter>
     <oddHeader>&amp;C&amp;G</oddHeader>
   </headerFooter>
-  <legacyDrawingHF r:id="rId2"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawingHF r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -2259,136 +2310,136 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
     </row>
     <row r="3" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="41" t="s">
+      <c r="A3" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="42"/>
-      <c r="C3" s="43" t="s">
+      <c r="B3" s="40"/>
+      <c r="C3" s="41" t="s">
         <v>51</v>
       </c>
-      <c r="D3" s="44"/>
-      <c r="E3" s="44"/>
-      <c r="F3" s="41" t="s">
+      <c r="D3" s="42"/>
+      <c r="E3" s="42"/>
+      <c r="F3" s="39" t="s">
         <v>32</v>
       </c>
-      <c r="G3" s="42"/>
-      <c r="H3" s="43" t="s">
+      <c r="G3" s="40"/>
+      <c r="H3" s="41" t="s">
         <v>52</v>
       </c>
-      <c r="I3" s="44"/>
-      <c r="J3" s="44"/>
-      <c r="K3" s="44"/>
-      <c r="L3" s="56"/>
-      <c r="M3" s="57"/>
+      <c r="I3" s="42"/>
+      <c r="J3" s="42"/>
+      <c r="K3" s="42"/>
+      <c r="L3" s="49"/>
+      <c r="M3" s="50"/>
     </row>
     <row r="4" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="41" t="s">
+      <c r="A4" s="39" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="42"/>
-      <c r="C4" s="43" t="s">
+      <c r="B4" s="40"/>
+      <c r="C4" s="41" t="s">
         <v>50</v>
       </c>
-      <c r="D4" s="44"/>
-      <c r="E4" s="44"/>
-      <c r="F4" s="41" t="s">
+      <c r="D4" s="42"/>
+      <c r="E4" s="42"/>
+      <c r="F4" s="39" t="s">
         <v>27</v>
       </c>
-      <c r="G4" s="42"/>
-      <c r="H4" s="43" t="s">
+      <c r="G4" s="40"/>
+      <c r="H4" s="41" t="s">
         <v>53</v>
       </c>
-      <c r="I4" s="44"/>
-      <c r="J4" s="44"/>
-      <c r="K4" s="44"/>
-      <c r="L4" s="58"/>
-      <c r="M4" s="59"/>
+      <c r="I4" s="42"/>
+      <c r="J4" s="42"/>
+      <c r="K4" s="42"/>
+      <c r="L4" s="51"/>
+      <c r="M4" s="52"/>
     </row>
     <row r="5" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="41" t="s">
+      <c r="A5" s="39" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="42"/>
-      <c r="C5" s="52"/>
-      <c r="D5" s="53"/>
-      <c r="E5" s="54"/>
-      <c r="F5" s="41" t="s">
+      <c r="B5" s="40"/>
+      <c r="C5" s="58"/>
+      <c r="D5" s="59"/>
+      <c r="E5" s="60"/>
+      <c r="F5" s="39" t="s">
         <v>33</v>
       </c>
-      <c r="G5" s="42"/>
-      <c r="H5" s="43" t="s">
+      <c r="G5" s="40"/>
+      <c r="H5" s="41" t="s">
         <v>54</v>
       </c>
-      <c r="I5" s="44"/>
-      <c r="J5" s="44"/>
-      <c r="K5" s="44"/>
-      <c r="L5" s="58"/>
-      <c r="M5" s="59"/>
+      <c r="I5" s="42"/>
+      <c r="J5" s="42"/>
+      <c r="K5" s="42"/>
+      <c r="L5" s="51"/>
+      <c r="M5" s="52"/>
     </row>
     <row r="6" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="41" t="s">
+      <c r="A6" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="42"/>
+      <c r="B6" s="40"/>
       <c r="C6" s="45" t="s">
         <v>56</v>
       </c>
-      <c r="D6" s="55"/>
+      <c r="D6" s="61"/>
       <c r="E6" s="46"/>
-      <c r="F6" s="41" t="s">
+      <c r="F6" s="39" t="s">
         <v>34</v>
       </c>
-      <c r="G6" s="42"/>
-      <c r="H6" s="43" t="s">
+      <c r="G6" s="40"/>
+      <c r="H6" s="41" t="s">
         <v>55</v>
       </c>
-      <c r="I6" s="44"/>
-      <c r="J6" s="44"/>
-      <c r="K6" s="44"/>
-      <c r="L6" s="58"/>
-      <c r="M6" s="59"/>
+      <c r="I6" s="42"/>
+      <c r="J6" s="42"/>
+      <c r="K6" s="42"/>
+      <c r="L6" s="51"/>
+      <c r="M6" s="52"/>
     </row>
     <row r="7" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="41" t="s">
+      <c r="A7" s="39" t="s">
         <v>39</v>
       </c>
-      <c r="B7" s="42"/>
-      <c r="C7" s="43">
+      <c r="B7" s="40"/>
+      <c r="C7" s="41">
         <v>12</v>
       </c>
-      <c r="D7" s="44"/>
-      <c r="E7" s="44"/>
-      <c r="F7" s="49" t="s">
+      <c r="D7" s="42"/>
+      <c r="E7" s="42"/>
+      <c r="F7" s="55" t="s">
         <v>40</v>
       </c>
-      <c r="G7" s="50"/>
-      <c r="H7" s="51" t="s">
+      <c r="G7" s="56"/>
+      <c r="H7" s="57" t="s">
         <v>57</v>
       </c>
-      <c r="I7" s="44"/>
-      <c r="J7" s="44"/>
-      <c r="K7" s="44"/>
-      <c r="L7" s="58"/>
-      <c r="M7" s="59"/>
+      <c r="I7" s="42"/>
+      <c r="J7" s="42"/>
+      <c r="K7" s="42"/>
+      <c r="L7" s="51"/>
+      <c r="M7" s="52"/>
     </row>
     <row r="8" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="41" t="s">
+      <c r="A8" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="42"/>
-      <c r="C8" s="43" t="s">
+      <c r="B8" s="40"/>
+      <c r="C8" s="41" t="s">
         <v>58</v>
       </c>
-      <c r="D8" s="44"/>
-      <c r="E8" s="44"/>
+      <c r="D8" s="42"/>
+      <c r="E8" s="42"/>
       <c r="F8" s="9" t="s">
         <v>35</v>
       </c>
@@ -2403,19 +2454,19 @@
         <v>47098</v>
       </c>
       <c r="K8" s="46"/>
-      <c r="L8" s="58"/>
-      <c r="M8" s="59"/>
+      <c r="L8" s="51"/>
+      <c r="M8" s="52"/>
     </row>
     <row r="9" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="41" t="s">
+      <c r="A9" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="42"/>
-      <c r="C9" s="43" t="s">
+      <c r="B9" s="40"/>
+      <c r="C9" s="41" t="s">
         <v>59</v>
       </c>
-      <c r="D9" s="44"/>
-      <c r="E9" s="44"/>
+      <c r="D9" s="42"/>
+      <c r="E9" s="42"/>
       <c r="F9" s="9" t="s">
         <v>35</v>
       </c>
@@ -2430,34 +2481,34 @@
         <v>47101</v>
       </c>
       <c r="K9" s="46"/>
-      <c r="L9" s="60"/>
-      <c r="M9" s="61"/>
+      <c r="L9" s="53"/>
+      <c r="M9" s="54"/>
     </row>
     <row r="10" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="41" t="s">
+      <c r="A10" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="B10" s="42"/>
+      <c r="B10" s="40"/>
       <c r="C10" s="47"/>
-      <c r="D10" s="44"/>
-      <c r="E10" s="44"/>
+      <c r="D10" s="42"/>
+      <c r="E10" s="42"/>
       <c r="F10" s="9" t="s">
         <v>35</v>
       </c>
       <c r="G10" s="48"/>
-      <c r="H10" s="43"/>
+      <c r="H10" s="41"/>
       <c r="I10" s="5"/>
       <c r="J10" s="5"/>
       <c r="K10" s="5"/>
     </row>
     <row r="12" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="28" t="s">
+      <c r="A12" s="31" t="s">
         <v>28</v>
       </c>
-      <c r="B12" s="28"/>
-      <c r="C12" s="28"/>
-      <c r="D12" s="28"/>
-      <c r="E12" s="28"/>
+      <c r="B12" s="31"/>
+      <c r="C12" s="31"/>
+      <c r="D12" s="31"/>
+      <c r="E12" s="31"/>
     </row>
     <row r="14" spans="1:13" s="7" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="36" t="s">
@@ -2470,10 +2521,10 @@
         <v>30</v>
       </c>
       <c r="F14" s="26"/>
-      <c r="G14" s="39" t="s">
+      <c r="G14" s="43" t="s">
         <v>31</v>
       </c>
-      <c r="H14" s="40"/>
+      <c r="H14" s="44"/>
       <c r="I14" s="26" t="s">
         <v>11</v>
       </c>
@@ -2527,12 +2578,12 @@
       <c r="M16" s="18"/>
     </row>
     <row r="18" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="28" t="s">
+      <c r="A18" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="B18" s="28"/>
-      <c r="C18" s="28"/>
-      <c r="D18" s="28"/>
+      <c r="B18" s="31"/>
+      <c r="C18" s="31"/>
+      <c r="D18" s="31"/>
     </row>
     <row r="20" spans="1:13" s="3" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="26" t="s">
@@ -2540,20 +2591,20 @@
       </c>
       <c r="B20" s="26"/>
       <c r="C20" s="26"/>
-      <c r="D20" s="24" t="s">
+      <c r="D20" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="E20" s="24"/>
-      <c r="F20" s="24"/>
-      <c r="G20" s="24"/>
-      <c r="H20" s="24"/>
-      <c r="I20" s="24" t="s">
+      <c r="E20" s="22"/>
+      <c r="F20" s="22"/>
+      <c r="G20" s="22"/>
+      <c r="H20" s="22"/>
+      <c r="I20" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="J20" s="24"/>
-      <c r="K20" s="24"/>
-      <c r="L20" s="24"/>
-      <c r="M20" s="24"/>
+      <c r="J20" s="22"/>
+      <c r="K20" s="22"/>
+      <c r="L20" s="22"/>
+      <c r="M20" s="22"/>
     </row>
     <row r="21" spans="1:13" s="3" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="26"/>
@@ -2906,149 +2957,149 @@
       <c r="M42" s="8"/>
     </row>
     <row r="44" spans="1:13" ht="26.4" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="28" t="s">
+      <c r="A44" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="B44" s="28"/>
-      <c r="C44" s="28"/>
-      <c r="D44" s="28"/>
-      <c r="E44" s="28"/>
+      <c r="B44" s="31"/>
+      <c r="C44" s="31"/>
+      <c r="D44" s="31"/>
+      <c r="E44" s="31"/>
     </row>
     <row r="46" spans="1:13" s="3" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="24" t="s">
+      <c r="A46" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="B46" s="24"/>
-      <c r="C46" s="24"/>
-      <c r="D46" s="24"/>
-      <c r="E46" s="24" t="s">
+      <c r="B46" s="22"/>
+      <c r="C46" s="22"/>
+      <c r="D46" s="22"/>
+      <c r="E46" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="F46" s="24"/>
-      <c r="G46" s="24" t="s">
+      <c r="F46" s="22"/>
+      <c r="G46" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="H46" s="24"/>
-      <c r="I46" s="24"/>
-      <c r="J46" s="24" t="s">
+      <c r="H46" s="22"/>
+      <c r="I46" s="22"/>
+      <c r="J46" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="K46" s="24"/>
-      <c r="L46" s="24" t="s">
+      <c r="K46" s="22"/>
+      <c r="L46" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="M46" s="24"/>
+      <c r="M46" s="22"/>
     </row>
     <row r="47" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="29" t="s">
+      <c r="A47" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="B47" s="29"/>
-      <c r="C47" s="29"/>
-      <c r="D47" s="29"/>
-      <c r="E47" s="30"/>
-      <c r="F47" s="30"/>
-      <c r="G47" s="31"/>
-      <c r="H47" s="31"/>
-      <c r="I47" s="31"/>
-      <c r="J47" s="32"/>
-      <c r="K47" s="32"/>
-      <c r="L47" s="32"/>
-      <c r="M47" s="32"/>
+      <c r="B47" s="28"/>
+      <c r="C47" s="28"/>
+      <c r="D47" s="28"/>
+      <c r="E47" s="32"/>
+      <c r="F47" s="32"/>
+      <c r="G47" s="29"/>
+      <c r="H47" s="29"/>
+      <c r="I47" s="29"/>
+      <c r="J47" s="30"/>
+      <c r="K47" s="30"/>
+      <c r="L47" s="30"/>
+      <c r="M47" s="30"/>
     </row>
     <row r="48" spans="1:13" ht="40.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="29" t="s">
+      <c r="A48" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="B48" s="29"/>
-      <c r="C48" s="29"/>
-      <c r="D48" s="29"/>
-      <c r="E48" s="31"/>
-      <c r="F48" s="31"/>
-      <c r="G48" s="31"/>
-      <c r="H48" s="31"/>
-      <c r="I48" s="31"/>
-      <c r="J48" s="32"/>
-      <c r="K48" s="32"/>
-      <c r="L48" s="32"/>
-      <c r="M48" s="32"/>
+      <c r="B48" s="28"/>
+      <c r="C48" s="28"/>
+      <c r="D48" s="28"/>
+      <c r="E48" s="29"/>
+      <c r="F48" s="29"/>
+      <c r="G48" s="29"/>
+      <c r="H48" s="29"/>
+      <c r="I48" s="29"/>
+      <c r="J48" s="30"/>
+      <c r="K48" s="30"/>
+      <c r="L48" s="30"/>
+      <c r="M48" s="30"/>
     </row>
     <row r="49" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="28" t="s">
+      <c r="A49" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="B49" s="28"/>
-      <c r="C49" s="28"/>
-      <c r="D49" s="28"/>
+      <c r="B49" s="31"/>
+      <c r="C49" s="31"/>
+      <c r="D49" s="31"/>
     </row>
     <row r="51" spans="1:13" s="3" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="24" t="s">
+      <c r="A51" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="B51" s="24"/>
-      <c r="C51" s="24"/>
-      <c r="D51" s="24"/>
-      <c r="E51" s="24" t="s">
+      <c r="B51" s="22"/>
+      <c r="C51" s="22"/>
+      <c r="D51" s="22"/>
+      <c r="E51" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="F51" s="24"/>
-      <c r="G51" s="24"/>
-      <c r="H51" s="24" t="s">
+      <c r="F51" s="22"/>
+      <c r="G51" s="22"/>
+      <c r="H51" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="I51" s="24"/>
-      <c r="J51" s="24"/>
-      <c r="K51" s="24" t="s">
+      <c r="I51" s="22"/>
+      <c r="J51" s="22"/>
+      <c r="K51" s="22" t="s">
         <v>37</v>
       </c>
-      <c r="L51" s="24"/>
-      <c r="M51" s="24"/>
+      <c r="L51" s="22"/>
+      <c r="M51" s="22"/>
     </row>
     <row r="52" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="23" t="s">
+      <c r="A52" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="B52" s="23"/>
-      <c r="C52" s="23"/>
-      <c r="D52" s="23"/>
-      <c r="E52" s="24" t="s">
+      <c r="B52" s="21"/>
+      <c r="C52" s="21"/>
+      <c r="D52" s="21"/>
+      <c r="E52" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="F52" s="24"/>
-      <c r="G52" s="24"/>
-      <c r="H52" s="24" t="s">
+      <c r="F52" s="22"/>
+      <c r="G52" s="22"/>
+      <c r="H52" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="I52" s="24"/>
-      <c r="J52" s="24"/>
-      <c r="K52" s="24" t="s">
+      <c r="I52" s="22"/>
+      <c r="J52" s="22"/>
+      <c r="K52" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="L52" s="24"/>
-      <c r="M52" s="24"/>
+      <c r="L52" s="22"/>
+      <c r="M52" s="22"/>
     </row>
     <row r="53" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="23" t="s">
+      <c r="A53" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="B53" s="23"/>
-      <c r="C53" s="23"/>
-      <c r="D53" s="23"/>
-      <c r="E53" s="24" t="s">
+      <c r="B53" s="21"/>
+      <c r="C53" s="21"/>
+      <c r="D53" s="21"/>
+      <c r="E53" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="F53" s="24"/>
-      <c r="G53" s="24"/>
-      <c r="H53" s="24" t="s">
+      <c r="F53" s="22"/>
+      <c r="G53" s="22"/>
+      <c r="H53" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="I53" s="24"/>
-      <c r="J53" s="24"/>
-      <c r="K53" s="24" t="s">
+      <c r="I53" s="22"/>
+      <c r="J53" s="22"/>
+      <c r="K53" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="L53" s="24"/>
-      <c r="M53" s="24"/>
+      <c r="L53" s="22"/>
+      <c r="M53" s="22"/>
     </row>
     <row r="55" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="25" t="s">
@@ -3111,8 +3162,8 @@
       <c r="G58" s="15"/>
       <c r="H58" s="19"/>
       <c r="I58" s="20"/>
-      <c r="J58" s="21"/>
-      <c r="K58" s="22"/>
+      <c r="J58" s="23"/>
+      <c r="K58" s="24"/>
       <c r="L58" s="15"/>
       <c r="M58" s="15"/>
     </row>
@@ -3489,7 +3540,7 @@
     <mergeCell ref="A52:D52"/>
     <mergeCell ref="B60:C60"/>
     <mergeCell ref="H60:I60"/>
-    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="B62:C62"/>
     <mergeCell ref="H73:I73"/>
     <mergeCell ref="F35:G35"/>
     <mergeCell ref="F36:G36"/>
@@ -3498,31 +3549,10 @@
     <mergeCell ref="F39:G39"/>
     <mergeCell ref="F40:G40"/>
     <mergeCell ref="H58:I58"/>
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="A29:C29"/>
-    <mergeCell ref="A30:C30"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="A33:C33"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="F23:G23"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="I16:J16"/>
-    <mergeCell ref="F26:G26"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="F32:G32"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="A24:C24"/>
     <mergeCell ref="H66:I66"/>
+    <mergeCell ref="H61:I61"/>
+    <mergeCell ref="H62:I62"/>
+    <mergeCell ref="H57:I57"/>
     <mergeCell ref="J66:K66"/>
     <mergeCell ref="J57:K57"/>
     <mergeCell ref="A20:C21"/>
@@ -3546,6 +3576,7 @@
     <mergeCell ref="J65:K65"/>
     <mergeCell ref="A34:C34"/>
     <mergeCell ref="A35:C35"/>
+    <mergeCell ref="B61:C61"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A12:E12"/>
     <mergeCell ref="A18:D18"/>
@@ -3607,13 +3638,6 @@
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="J9:K9"/>
     <mergeCell ref="J8:K8"/>
-    <mergeCell ref="B61:C61"/>
-    <mergeCell ref="H61:I61"/>
-    <mergeCell ref="B62:C62"/>
-    <mergeCell ref="H62:I62"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="G46:I46"/>
-    <mergeCell ref="E46:F46"/>
     <mergeCell ref="J46:K46"/>
     <mergeCell ref="L46:M46"/>
     <mergeCell ref="I14:J14"/>
@@ -3623,7 +3647,21 @@
     <mergeCell ref="I21:J21"/>
     <mergeCell ref="E16:F16"/>
     <mergeCell ref="L16:M16"/>
-    <mergeCell ref="H57:I57"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="F23:G23"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="I16:J16"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="F31:G31"/>
     <mergeCell ref="A36:C36"/>
     <mergeCell ref="A37:C37"/>
     <mergeCell ref="A38:C38"/>
@@ -3631,6 +3669,19 @@
     <mergeCell ref="A40:C40"/>
     <mergeCell ref="A41:C41"/>
     <mergeCell ref="A42:C42"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="G46:I46"/>
+    <mergeCell ref="E46:F46"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="F34:G34"/>
   </mergeCells>
   <pageMargins left="0.31496062992125984" right="0.31496062992125984" top="1.1811023622047245" bottom="0.51181102362204722" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="8" scale="94" fitToHeight="0" orientation="portrait" r:id="rId1"/>

</xml_diff>